<commit_message>
Add load_results_temp() + temp Excel file
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/00_functions/test_data/emission_factors_fossil_grid.xlsx
+++ b/Spine_Projects/03_output_data/00_functions/test_data/emission_factors_fossil_grid.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10208"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC071FE1-0BB4-CB4C-9EC8-8E38C3170F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F188BFD-58A3-B641-99AE-A0FD974D4D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Emmission_Factors_Fossils" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>Upper range</t>
   </si>
@@ -73,7 +73,7 @@
     <t>Jet_Fuel</t>
   </si>
   <si>
-    <t>DK1</t>
+    <t>DK</t>
   </si>
   <si>
     <t>DK2</t>
@@ -113,12 +113,6 @@
   </si>
   <si>
     <t>DE</t>
-  </si>
-  <si>
-    <t>478,5</t>
-  </si>
-  <si>
-    <t>411,5</t>
   </si>
 </sst>
 </file>
@@ -808,8 +802,8 @@
       <c r="A4">
         <v>2020</v>
       </c>
-      <c r="B4" t="s">
-        <v>28</v>
+      <c r="B4">
+        <v>478.5</v>
       </c>
       <c r="C4">
         <f t="shared" si="1"/>
@@ -868,8 +862,8 @@
       <c r="A5">
         <v>2021</v>
       </c>
-      <c r="B5" t="s">
-        <v>29</v>
+      <c r="B5">
+        <v>411.5</v>
       </c>
       <c r="C5">
         <f t="shared" si="1"/>

</xml_diff>